<commit_message>
MAJ pipeline 2026-07-31 13:47
</commit_message>
<xml_diff>
--- a/jira_export_2026-07-31.xlsx
+++ b/jira_export_2026-07-31.xlsx
@@ -14327,7 +14327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -14353,7 +14353,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tickets 'Matériel GEODP' clôturés ce mois — 8 ligne(s)</t>
+          <t>Tickets 'Matériel GEODP' clôturés ce mois — 9 ligne(s)</t>
         </is>
       </c>
     </row>
@@ -14736,22 +14736,22 @@
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-32732</t>
+          <t>PDMDEP-33597</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>[MAIRIE DE LA SENTINELLE] - Acquisition Geodp Caisse</t>
+          <t>[Commune de Trets] - Ajout d'un Module Caisse sur GEODP avec paiement CB</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>MAIRIE DE LA SENTINELLE</t>
+          <t>Commune de Trets</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Acquisition Geodp Caisse</t>
+          <t>Ajout d'un Module Caisse sur GEODP avec paiement CB</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
@@ -14766,7 +14766,7 @@
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>Nouveau déploiement</t>
+          <t>Vente additionnelle</t>
         </is>
       </c>
       <c r="H11" s="12" t="n">
@@ -14774,12 +14774,12 @@
       </c>
       <c r="I11" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-32739</t>
+          <t>PDMDEP-33603</t>
         </is>
       </c>
       <c r="J11" s="12" t="inlineStr">
         <is>
-          <t>00163790</t>
+          <t>00168996</t>
         </is>
       </c>
       <c r="K11" s="13" t="n">
@@ -14789,73 +14789,126 @@
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
+          <t>PDMDEP-32732</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>[MAIRIE DE LA SENTINELLE] - Acquisition Geodp Caisse</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>MAIRIE DE LA SENTINELLE</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>Acquisition Geodp Caisse</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>GEODP</t>
+        </is>
+      </c>
+      <c r="F12" s="15" t="inlineStr">
+        <is>
+          <t>Projet</t>
+        </is>
+      </c>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>Nouveau déploiement</t>
+        </is>
+      </c>
+      <c r="H12" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="15" t="inlineStr">
+        <is>
+          <t>PDMDEP-32739</t>
+        </is>
+      </c>
+      <c r="J12" s="15" t="inlineStr">
+        <is>
+          <t>00163790</t>
+        </is>
+      </c>
+      <c r="K12" s="16" t="n">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
           <t>PDMDEP-32152</t>
         </is>
       </c>
-      <c r="B12" s="15" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">[COMMUNE DE CAVAILLON] - Migration GeODP Placier + CB + Formation sur site </t>
         </is>
       </c>
-      <c r="C12" s="15" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>COMMUNE DE CAVAILLON</t>
         </is>
       </c>
-      <c r="D12" s="15" t="inlineStr">
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Migration GeODP Placier + CB + Formation sur site </t>
         </is>
       </c>
-      <c r="E12" s="15" t="inlineStr">
+      <c r="E13" s="12" t="inlineStr">
         <is>
           <t>GEODP</t>
         </is>
       </c>
-      <c r="F12" s="15" t="inlineStr">
-        <is>
-          <t>Projet</t>
-        </is>
-      </c>
-      <c r="G12" s="15" t="inlineStr">
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>Projet</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="inlineStr">
         <is>
           <t>Migration</t>
         </is>
       </c>
-      <c r="H12" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="15" t="inlineStr">
+      <c r="H13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
         <is>
           <t>PDMDEP-32159</t>
         </is>
       </c>
-      <c r="J12" s="15" t="inlineStr">
+      <c r="J13" s="12" t="inlineStr">
         <is>
           <t>00160662</t>
         </is>
       </c>
-      <c r="K12" s="16" t="n">
+      <c r="K13" s="13" t="n">
         <v>1711.5</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B13" s="18" t="inlineStr"/>
-      <c r="C13" s="18" t="inlineStr"/>
-      <c r="D13" s="18" t="inlineStr"/>
-      <c r="E13" s="18" t="inlineStr"/>
-      <c r="F13" s="18" t="inlineStr"/>
-      <c r="G13" s="18" t="inlineStr"/>
-      <c r="H13" s="18" t="inlineStr"/>
-      <c r="I13" s="18" t="inlineStr"/>
-      <c r="J13" s="18" t="inlineStr"/>
-      <c r="K13" s="19" t="n">
-        <v>8231.5</v>
+      <c r="B14" s="18" t="inlineStr"/>
+      <c r="C14" s="18" t="inlineStr"/>
+      <c r="D14" s="18" t="inlineStr"/>
+      <c r="E14" s="18" t="inlineStr"/>
+      <c r="F14" s="18" t="inlineStr"/>
+      <c r="G14" s="18" t="inlineStr"/>
+      <c r="H14" s="18" t="inlineStr"/>
+      <c r="I14" s="18" t="inlineStr"/>
+      <c r="J14" s="18" t="inlineStr"/>
+      <c r="K14" s="19" t="n">
+        <v>9046.5</v>
       </c>
     </row>
   </sheetData>
@@ -14869,6 +14922,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>